<commit_message>
Update gitignore + remove logs from tracking + fix BO2+agent collection data
</commit_message>
<xml_diff>
--- a/BO4/dataset_BO4_contrats_final.xlsx
+++ b/BO4/dataset_BO4_contrats_final.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contrats_BO4" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Contrats_BO4" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Ajout datasets + embeddings
</commit_message>
<xml_diff>
--- a/BO4/dataset_BO4_contrats_final.xlsx
+++ b/BO4/dataset_BO4_contrats_final.xlsx
@@ -1054,7 +1054,7 @@
         <v>143</v>
       </c>
       <c r="M5" t="n">
-        <v>835</v>
+        <v>848</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
         <v>143</v>
       </c>
       <c r="M6" t="n">
-        <v>835</v>
+        <v>848</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
@@ -1310,7 +1310,7 @@
         <v>143</v>
       </c>
       <c r="M7" t="n">
-        <v>835</v>
+        <v>848</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
@@ -1438,7 +1438,7 @@
         <v>143</v>
       </c>
       <c r="M8" t="n">
-        <v>837</v>
+        <v>850</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
@@ -1566,7 +1566,7 @@
         <v>143</v>
       </c>
       <c r="M9" t="n">
-        <v>836</v>
+        <v>849</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
@@ -1694,7 +1694,7 @@
         <v>143</v>
       </c>
       <c r="M10" t="n">
-        <v>835</v>
+        <v>848</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
@@ -1822,7 +1822,7 @@
         <v>133</v>
       </c>
       <c r="M11" t="n">
-        <v>778</v>
+        <v>790</v>
       </c>
       <c r="N11" t="inlineStr">
         <is>
@@ -1950,7 +1950,7 @@
         <v>143</v>
       </c>
       <c r="M12" t="n">
-        <v>835</v>
+        <v>848</v>
       </c>
       <c r="N12" t="inlineStr">
         <is>
@@ -2078,7 +2078,7 @@
         <v>133</v>
       </c>
       <c r="M13" t="n">
-        <v>778</v>
+        <v>790</v>
       </c>
       <c r="N13" t="inlineStr">
         <is>
@@ -2206,7 +2206,7 @@
         <v>143</v>
       </c>
       <c r="M14" t="n">
-        <v>836</v>
+        <v>849</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
@@ -2334,7 +2334,7 @@
         <v>143</v>
       </c>
       <c r="M15" t="n">
-        <v>835</v>
+        <v>848</v>
       </c>
       <c r="N15" t="inlineStr">
         <is>
@@ -2462,7 +2462,7 @@
         <v>143</v>
       </c>
       <c r="M16" t="n">
-        <v>835</v>
+        <v>848</v>
       </c>
       <c r="N16" t="inlineStr">
         <is>
@@ -2590,7 +2590,7 @@
         <v>143</v>
       </c>
       <c r="M17" t="n">
-        <v>835</v>
+        <v>848</v>
       </c>
       <c r="N17" t="inlineStr">
         <is>
@@ -2718,7 +2718,7 @@
         <v>143</v>
       </c>
       <c r="M18" t="n">
-        <v>835</v>
+        <v>848</v>
       </c>
       <c r="N18" t="inlineStr">
         <is>
@@ -2846,7 +2846,7 @@
         <v>143</v>
       </c>
       <c r="M19" t="n">
-        <v>836</v>
+        <v>849</v>
       </c>
       <c r="N19" t="inlineStr">
         <is>
@@ -2974,7 +2974,7 @@
         <v>143</v>
       </c>
       <c r="M20" t="n">
-        <v>837</v>
+        <v>850</v>
       </c>
       <c r="N20" t="inlineStr">
         <is>
@@ -3102,7 +3102,7 @@
         <v>143</v>
       </c>
       <c r="M21" t="n">
-        <v>836</v>
+        <v>849</v>
       </c>
       <c r="N21" t="inlineStr">
         <is>
@@ -3230,7 +3230,7 @@
         <v>143</v>
       </c>
       <c r="M22" t="n">
-        <v>833</v>
+        <v>846</v>
       </c>
       <c r="N22" t="inlineStr">
         <is>
@@ -3358,7 +3358,7 @@
         <v>143</v>
       </c>
       <c r="M23" t="n">
-        <v>836</v>
+        <v>849</v>
       </c>
       <c r="N23" t="inlineStr">
         <is>
@@ -3486,7 +3486,7 @@
         <v>143</v>
       </c>
       <c r="M24" t="n">
-        <v>837</v>
+        <v>850</v>
       </c>
       <c r="N24" t="inlineStr">
         <is>
@@ -3614,7 +3614,7 @@
         <v>143</v>
       </c>
       <c r="M25" t="n">
-        <v>836</v>
+        <v>849</v>
       </c>
       <c r="N25" t="inlineStr">
         <is>
@@ -3742,7 +3742,7 @@
         <v>143</v>
       </c>
       <c r="M26" t="n">
-        <v>837</v>
+        <v>850</v>
       </c>
       <c r="N26" t="inlineStr">
         <is>
@@ -3870,7 +3870,7 @@
         <v>143</v>
       </c>
       <c r="M27" t="n">
-        <v>836</v>
+        <v>849</v>
       </c>
       <c r="N27" t="inlineStr">
         <is>
@@ -3998,7 +3998,7 @@
         <v>133</v>
       </c>
       <c r="M28" t="n">
-        <v>778</v>
+        <v>790</v>
       </c>
       <c r="N28" t="inlineStr">
         <is>
@@ -4126,7 +4126,7 @@
         <v>143</v>
       </c>
       <c r="M29" t="n">
-        <v>837</v>
+        <v>850</v>
       </c>
       <c r="N29" t="inlineStr">
         <is>
@@ -4254,7 +4254,7 @@
         <v>143</v>
       </c>
       <c r="M30" t="n">
-        <v>837</v>
+        <v>850</v>
       </c>
       <c r="N30" t="inlineStr">
         <is>
@@ -4382,7 +4382,7 @@
         <v>143</v>
       </c>
       <c r="M31" t="n">
-        <v>835</v>
+        <v>848</v>
       </c>
       <c r="N31" t="inlineStr">
         <is>
@@ -4510,7 +4510,7 @@
         <v>143</v>
       </c>
       <c r="M32" t="n">
-        <v>836</v>
+        <v>849</v>
       </c>
       <c r="N32" t="inlineStr">
         <is>
@@ -4638,7 +4638,7 @@
         <v>149</v>
       </c>
       <c r="M33" t="n">
-        <v>881</v>
+        <v>895</v>
       </c>
       <c r="N33" t="inlineStr">
         <is>
@@ -4766,7 +4766,7 @@
         <v>149</v>
       </c>
       <c r="M34" t="n">
-        <v>881</v>
+        <v>895</v>
       </c>
       <c r="N34" t="inlineStr">
         <is>
@@ -4894,7 +4894,7 @@
         <v>149</v>
       </c>
       <c r="M35" t="n">
-        <v>881</v>
+        <v>895</v>
       </c>
       <c r="N35" t="inlineStr">
         <is>
@@ -5022,7 +5022,7 @@
         <v>149</v>
       </c>
       <c r="M36" t="n">
-        <v>879</v>
+        <v>893</v>
       </c>
       <c r="N36" t="inlineStr">
         <is>
@@ -5150,7 +5150,7 @@
         <v>149</v>
       </c>
       <c r="M37" t="n">
-        <v>879</v>
+        <v>893</v>
       </c>
       <c r="N37" t="inlineStr">
         <is>
@@ -5278,7 +5278,7 @@
         <v>149</v>
       </c>
       <c r="M38" t="n">
-        <v>885</v>
+        <v>899</v>
       </c>
       <c r="N38" t="inlineStr">
         <is>
@@ -5406,7 +5406,7 @@
         <v>149</v>
       </c>
       <c r="M39" t="n">
-        <v>881</v>
+        <v>895</v>
       </c>
       <c r="N39" t="inlineStr">
         <is>
@@ -5534,7 +5534,7 @@
         <v>149</v>
       </c>
       <c r="M40" t="n">
-        <v>883</v>
+        <v>897</v>
       </c>
       <c r="N40" t="inlineStr">
         <is>
@@ -5662,7 +5662,7 @@
         <v>149</v>
       </c>
       <c r="M41" t="n">
-        <v>881</v>
+        <v>895</v>
       </c>
       <c r="N41" t="inlineStr">
         <is>
@@ -5790,7 +5790,7 @@
         <v>149</v>
       </c>
       <c r="M42" t="n">
-        <v>879</v>
+        <v>893</v>
       </c>
       <c r="N42" t="inlineStr">
         <is>
@@ -5918,7 +5918,7 @@
         <v>149</v>
       </c>
       <c r="M43" t="n">
-        <v>881</v>
+        <v>895</v>
       </c>
       <c r="N43" t="inlineStr">
         <is>
@@ -6046,7 +6046,7 @@
         <v>149</v>
       </c>
       <c r="M44" t="n">
-        <v>881</v>
+        <v>895</v>
       </c>
       <c r="N44" t="inlineStr">
         <is>
@@ -6174,7 +6174,7 @@
         <v>149</v>
       </c>
       <c r="M45" t="n">
-        <v>883</v>
+        <v>897</v>
       </c>
       <c r="N45" t="inlineStr">
         <is>
@@ -6302,7 +6302,7 @@
         <v>149</v>
       </c>
       <c r="M46" t="n">
-        <v>880</v>
+        <v>894</v>
       </c>
       <c r="N46" t="inlineStr">
         <is>
@@ -6430,7 +6430,7 @@
         <v>149</v>
       </c>
       <c r="M47" t="n">
-        <v>883</v>
+        <v>897</v>
       </c>
       <c r="N47" t="inlineStr">
         <is>
@@ -6558,7 +6558,7 @@
         <v>149</v>
       </c>
       <c r="M48" t="n">
-        <v>880</v>
+        <v>894</v>
       </c>
       <c r="N48" t="inlineStr">
         <is>
@@ -6686,7 +6686,7 @@
         <v>149</v>
       </c>
       <c r="M49" t="n">
-        <v>882</v>
+        <v>896</v>
       </c>
       <c r="N49" t="inlineStr">
         <is>
@@ -6814,7 +6814,7 @@
         <v>149</v>
       </c>
       <c r="M50" t="n">
-        <v>882</v>
+        <v>896</v>
       </c>
       <c r="N50" t="inlineStr">
         <is>
@@ -6942,7 +6942,7 @@
         <v>149</v>
       </c>
       <c r="M51" t="n">
-        <v>880</v>
+        <v>894</v>
       </c>
       <c r="N51" t="inlineStr">
         <is>
@@ -7070,7 +7070,7 @@
         <v>149</v>
       </c>
       <c r="M52" t="n">
-        <v>881</v>
+        <v>895</v>
       </c>
       <c r="N52" t="inlineStr">
         <is>
@@ -7198,7 +7198,7 @@
         <v>149</v>
       </c>
       <c r="M53" t="n">
-        <v>879</v>
+        <v>893</v>
       </c>
       <c r="N53" t="inlineStr">
         <is>
@@ -7326,7 +7326,7 @@
         <v>149</v>
       </c>
       <c r="M54" t="n">
-        <v>882</v>
+        <v>896</v>
       </c>
       <c r="N54" t="inlineStr">
         <is>
@@ -7454,7 +7454,7 @@
         <v>149</v>
       </c>
       <c r="M55" t="n">
-        <v>881</v>
+        <v>895</v>
       </c>
       <c r="N55" t="inlineStr">
         <is>
@@ -7582,7 +7582,7 @@
         <v>149</v>
       </c>
       <c r="M56" t="n">
-        <v>881</v>
+        <v>895</v>
       </c>
       <c r="N56" t="inlineStr">
         <is>
@@ -7710,7 +7710,7 @@
         <v>149</v>
       </c>
       <c r="M57" t="n">
-        <v>881</v>
+        <v>895</v>
       </c>
       <c r="N57" t="inlineStr">
         <is>
@@ -7838,7 +7838,7 @@
         <v>149</v>
       </c>
       <c r="M58" t="n">
-        <v>881</v>
+        <v>895</v>
       </c>
       <c r="N58" t="inlineStr">
         <is>
@@ -7966,7 +7966,7 @@
         <v>149</v>
       </c>
       <c r="M59" t="n">
-        <v>881</v>
+        <v>895</v>
       </c>
       <c r="N59" t="inlineStr">
         <is>
@@ -8094,7 +8094,7 @@
         <v>149</v>
       </c>
       <c r="M60" t="n">
-        <v>881</v>
+        <v>895</v>
       </c>
       <c r="N60" t="inlineStr">
         <is>
@@ -8222,7 +8222,7 @@
         <v>149</v>
       </c>
       <c r="M61" t="n">
-        <v>883</v>
+        <v>897</v>
       </c>
       <c r="N61" t="inlineStr">
         <is>
@@ -8350,7 +8350,7 @@
         <v>416</v>
       </c>
       <c r="M62" t="n">
-        <v>2325</v>
+        <v>2346</v>
       </c>
       <c r="N62" t="inlineStr">
         <is>
@@ -8478,7 +8478,7 @@
         <v>416</v>
       </c>
       <c r="M63" t="n">
-        <v>2327</v>
+        <v>2348</v>
       </c>
       <c r="N63" t="inlineStr">
         <is>
@@ -8606,7 +8606,7 @@
         <v>416</v>
       </c>
       <c r="M64" t="n">
-        <v>2329</v>
+        <v>2350</v>
       </c>
       <c r="N64" t="inlineStr">
         <is>
@@ -8734,7 +8734,7 @@
         <v>416</v>
       </c>
       <c r="M65" t="n">
-        <v>2324</v>
+        <v>2345</v>
       </c>
       <c r="N65" t="inlineStr">
         <is>
@@ -8862,7 +8862,7 @@
         <v>416</v>
       </c>
       <c r="M66" t="n">
-        <v>2324</v>
+        <v>2345</v>
       </c>
       <c r="N66" t="inlineStr">
         <is>
@@ -8990,7 +8990,7 @@
         <v>416</v>
       </c>
       <c r="M67" t="n">
-        <v>2325</v>
+        <v>2346</v>
       </c>
       <c r="N67" t="inlineStr">
         <is>
@@ -9118,7 +9118,7 @@
         <v>416</v>
       </c>
       <c r="M68" t="n">
-        <v>2324</v>
+        <v>2345</v>
       </c>
       <c r="N68" t="inlineStr">
         <is>
@@ -9246,7 +9246,7 @@
         <v>416</v>
       </c>
       <c r="M69" t="n">
-        <v>2326</v>
+        <v>2347</v>
       </c>
       <c r="N69" t="inlineStr">
         <is>
@@ -9374,7 +9374,7 @@
         <v>181</v>
       </c>
       <c r="M70" t="n">
-        <v>1053</v>
+        <v>1066</v>
       </c>
       <c r="N70" t="inlineStr">
         <is>
@@ -9502,7 +9502,7 @@
         <v>135</v>
       </c>
       <c r="M71" t="n">
-        <v>820</v>
+        <v>834</v>
       </c>
       <c r="N71" t="inlineStr">
         <is>
@@ -9630,7 +9630,7 @@
         <v>135</v>
       </c>
       <c r="M72" t="n">
-        <v>818</v>
+        <v>832</v>
       </c>
       <c r="N72" t="inlineStr">
         <is>
@@ -9758,7 +9758,7 @@
         <v>185</v>
       </c>
       <c r="M73" t="n">
-        <v>1070</v>
+        <v>1083</v>
       </c>
       <c r="N73" t="inlineStr">
         <is>
@@ -9886,7 +9886,7 @@
         <v>294</v>
       </c>
       <c r="M74" t="n">
-        <v>1783</v>
+        <v>1801</v>
       </c>
       <c r="N74" t="inlineStr">
         <is>
@@ -10014,7 +10014,7 @@
         <v>184</v>
       </c>
       <c r="M75" t="n">
-        <v>1070</v>
+        <v>1083</v>
       </c>
       <c r="N75" t="inlineStr">
         <is>
@@ -10142,7 +10142,7 @@
         <v>150</v>
       </c>
       <c r="M76" t="n">
-        <v>988</v>
+        <v>1001</v>
       </c>
       <c r="N76" t="inlineStr">
         <is>
@@ -10270,7 +10270,7 @@
         <v>138</v>
       </c>
       <c r="M77" t="n">
-        <v>872</v>
+        <v>883</v>
       </c>
       <c r="N77" t="inlineStr">
         <is>
@@ -10398,7 +10398,7 @@
         <v>291</v>
       </c>
       <c r="M78" t="n">
-        <v>1764</v>
+        <v>1782</v>
       </c>
       <c r="N78" t="inlineStr">
         <is>
@@ -10526,7 +10526,7 @@
         <v>294</v>
       </c>
       <c r="M79" t="n">
-        <v>1778</v>
+        <v>1796</v>
       </c>
       <c r="N79" t="inlineStr">
         <is>
@@ -10654,7 +10654,7 @@
         <v>294</v>
       </c>
       <c r="M80" t="n">
-        <v>1779</v>
+        <v>1797</v>
       </c>
       <c r="N80" t="inlineStr">
         <is>
@@ -10782,7 +10782,7 @@
         <v>150</v>
       </c>
       <c r="M81" t="n">
-        <v>985</v>
+        <v>998</v>
       </c>
       <c r="N81" t="inlineStr">
         <is>
@@ -10910,7 +10910,7 @@
         <v>135</v>
       </c>
       <c r="M82" t="n">
-        <v>819</v>
+        <v>833</v>
       </c>
       <c r="N82" t="inlineStr">
         <is>
@@ -11038,7 +11038,7 @@
         <v>165</v>
       </c>
       <c r="M83" t="n">
-        <v>963</v>
+        <v>975</v>
       </c>
       <c r="N83" t="inlineStr">
         <is>
@@ -11166,7 +11166,7 @@
         <v>141</v>
       </c>
       <c r="M84" t="n">
-        <v>886</v>
+        <v>897</v>
       </c>
       <c r="N84" t="inlineStr">
         <is>
@@ -11294,7 +11294,7 @@
         <v>135</v>
       </c>
       <c r="M85" t="n">
-        <v>817</v>
+        <v>831</v>
       </c>
       <c r="N85" t="inlineStr">
         <is>
@@ -11422,7 +11422,7 @@
         <v>294</v>
       </c>
       <c r="M86" t="n">
-        <v>1778</v>
+        <v>1796</v>
       </c>
       <c r="N86" t="inlineStr">
         <is>
@@ -11550,7 +11550,7 @@
         <v>135</v>
       </c>
       <c r="M87" t="n">
-        <v>815</v>
+        <v>829</v>
       </c>
       <c r="N87" t="inlineStr">
         <is>
@@ -11678,7 +11678,7 @@
         <v>135</v>
       </c>
       <c r="M88" t="n">
-        <v>818</v>
+        <v>832</v>
       </c>
       <c r="N88" t="inlineStr">
         <is>
@@ -11806,7 +11806,7 @@
         <v>184</v>
       </c>
       <c r="M89" t="n">
-        <v>1068</v>
+        <v>1081</v>
       </c>
       <c r="N89" t="inlineStr">
         <is>
@@ -11934,7 +11934,7 @@
         <v>147</v>
       </c>
       <c r="M90" t="n">
-        <v>970</v>
+        <v>983</v>
       </c>
       <c r="N90" t="inlineStr">
         <is>
@@ -12062,7 +12062,7 @@
         <v>184</v>
       </c>
       <c r="M91" t="n">
-        <v>1072</v>
+        <v>1085</v>
       </c>
       <c r="N91" t="inlineStr">
         <is>
@@ -12190,7 +12190,7 @@
         <v>151</v>
       </c>
       <c r="M92" t="n">
-        <v>988</v>
+        <v>1001</v>
       </c>
       <c r="N92" t="inlineStr">
         <is>
@@ -12318,7 +12318,7 @@
         <v>294</v>
       </c>
       <c r="M93" t="n">
-        <v>1780</v>
+        <v>1798</v>
       </c>
       <c r="N93" t="inlineStr">
         <is>
@@ -12446,7 +12446,7 @@
         <v>328</v>
       </c>
       <c r="M94" t="n">
-        <v>1915</v>
+        <v>1937</v>
       </c>
       <c r="N94" t="inlineStr">
         <is>
@@ -12574,7 +12574,7 @@
         <v>165</v>
       </c>
       <c r="M95" t="n">
-        <v>987</v>
+        <v>1000</v>
       </c>
       <c r="N95" t="inlineStr">
         <is>
@@ -12702,7 +12702,7 @@
         <v>329</v>
       </c>
       <c r="M96" t="n">
-        <v>1892</v>
+        <v>1910</v>
       </c>
       <c r="N96" t="inlineStr">
         <is>
@@ -12958,7 +12958,7 @@
         <v>329</v>
       </c>
       <c r="M98" t="n">
-        <v>1894</v>
+        <v>1912</v>
       </c>
       <c r="N98" t="inlineStr">
         <is>
@@ -13086,7 +13086,7 @@
         <v>326</v>
       </c>
       <c r="M99" t="n">
-        <v>1908</v>
+        <v>1930</v>
       </c>
       <c r="N99" t="inlineStr">
         <is>
@@ -13342,7 +13342,7 @@
         <v>189</v>
       </c>
       <c r="M101" t="n">
-        <v>1189</v>
+        <v>1203</v>
       </c>
       <c r="N101" t="inlineStr">
         <is>
@@ -13470,7 +13470,7 @@
         <v>151</v>
       </c>
       <c r="M102" t="n">
-        <v>935</v>
+        <v>947</v>
       </c>
       <c r="N102" t="inlineStr">
         <is>
@@ -13598,7 +13598,7 @@
         <v>329</v>
       </c>
       <c r="M103" t="n">
-        <v>1893</v>
+        <v>1911</v>
       </c>
       <c r="N103" t="inlineStr">
         <is>
@@ -13854,7 +13854,7 @@
         <v>165</v>
       </c>
       <c r="M105" t="n">
-        <v>987</v>
+        <v>1000</v>
       </c>
       <c r="N105" t="inlineStr">
         <is>
@@ -13982,7 +13982,7 @@
         <v>326</v>
       </c>
       <c r="M106" t="n">
-        <v>1909</v>
+        <v>1931</v>
       </c>
       <c r="N106" t="inlineStr">
         <is>
@@ -14110,7 +14110,7 @@
         <v>224</v>
       </c>
       <c r="M107" t="n">
-        <v>1325</v>
+        <v>1339</v>
       </c>
       <c r="N107" t="inlineStr">
         <is>
@@ -14238,7 +14238,7 @@
         <v>224</v>
       </c>
       <c r="M108" t="n">
-        <v>1323</v>
+        <v>1337</v>
       </c>
       <c r="N108" t="inlineStr">
         <is>
@@ -14366,7 +14366,7 @@
         <v>189</v>
       </c>
       <c r="M109" t="n">
-        <v>1189</v>
+        <v>1203</v>
       </c>
       <c r="N109" t="inlineStr">
         <is>
@@ -14494,7 +14494,7 @@
         <v>314</v>
       </c>
       <c r="M110" t="n">
-        <v>1812</v>
+        <v>1829</v>
       </c>
       <c r="N110" t="inlineStr">
         <is>
@@ -14750,7 +14750,7 @@
         <v>189</v>
       </c>
       <c r="M112" t="n">
-        <v>1186</v>
+        <v>1200</v>
       </c>
       <c r="N112" t="inlineStr">
         <is>
@@ -14878,7 +14878,7 @@
         <v>187</v>
       </c>
       <c r="M113" t="n">
-        <v>1180</v>
+        <v>1194</v>
       </c>
       <c r="N113" t="inlineStr">
         <is>
@@ -15134,7 +15134,7 @@
         <v>329</v>
       </c>
       <c r="M115" t="n">
-        <v>1896</v>
+        <v>1914</v>
       </c>
       <c r="N115" t="inlineStr">
         <is>
@@ -15262,7 +15262,7 @@
         <v>328</v>
       </c>
       <c r="M116" t="n">
-        <v>1915</v>
+        <v>1937</v>
       </c>
       <c r="N116" t="inlineStr">
         <is>
@@ -15390,7 +15390,7 @@
         <v>189</v>
       </c>
       <c r="M117" t="n">
-        <v>1185</v>
+        <v>1199</v>
       </c>
       <c r="N117" t="inlineStr">
         <is>
@@ -15518,7 +15518,7 @@
         <v>168</v>
       </c>
       <c r="M118" t="n">
-        <v>1000</v>
+        <v>1013</v>
       </c>
       <c r="N118" t="inlineStr">
         <is>
@@ -15646,7 +15646,7 @@
         <v>328</v>
       </c>
       <c r="M119" t="n">
-        <v>1915</v>
+        <v>1937</v>
       </c>
       <c r="N119" t="inlineStr">
         <is>
@@ -15774,7 +15774,7 @@
         <v>224</v>
       </c>
       <c r="M120" t="n">
-        <v>1323</v>
+        <v>1337</v>
       </c>
       <c r="N120" t="inlineStr">
         <is>
@@ -15902,7 +15902,7 @@
         <v>221</v>
       </c>
       <c r="M121" t="n">
-        <v>1309</v>
+        <v>1323</v>
       </c>
       <c r="N121" t="inlineStr">
         <is>
@@ -16030,7 +16030,7 @@
         <v>329</v>
       </c>
       <c r="M122" t="n">
-        <v>1896</v>
+        <v>1914</v>
       </c>
       <c r="N122" t="inlineStr">
         <is>
@@ -16158,7 +16158,7 @@
         <v>326</v>
       </c>
       <c r="M123" t="n">
-        <v>1911</v>
+        <v>1933</v>
       </c>
       <c r="N123" t="inlineStr">
         <is>
@@ -16286,7 +16286,7 @@
         <v>311</v>
       </c>
       <c r="M124" t="n">
-        <v>1827</v>
+        <v>1848</v>
       </c>
       <c r="N124" t="inlineStr">
         <is>
@@ -16414,7 +16414,7 @@
         <v>292</v>
       </c>
       <c r="M125" t="n">
-        <v>1702</v>
+        <v>1723</v>
       </c>
       <c r="N125" t="inlineStr">
         <is>
@@ -16542,7 +16542,7 @@
         <v>168</v>
       </c>
       <c r="M126" t="n">
-        <v>1000</v>
+        <v>1013</v>
       </c>
       <c r="N126" t="inlineStr">
         <is>
@@ -16670,7 +16670,7 @@
         <v>329</v>
       </c>
       <c r="M127" t="n">
-        <v>1895</v>
+        <v>1913</v>
       </c>
       <c r="N127" t="inlineStr">
         <is>
@@ -16798,7 +16798,7 @@
         <v>328</v>
       </c>
       <c r="M128" t="n">
-        <v>1916</v>
+        <v>1938</v>
       </c>
       <c r="N128" t="inlineStr">
         <is>
@@ -16926,7 +16926,7 @@
         <v>154</v>
       </c>
       <c r="M129" t="n">
-        <v>954</v>
+        <v>966</v>
       </c>
       <c r="N129" t="inlineStr">
         <is>
@@ -17054,7 +17054,7 @@
         <v>165</v>
       </c>
       <c r="M130" t="n">
-        <v>987</v>
+        <v>1000</v>
       </c>
       <c r="N130" t="inlineStr">
         <is>
@@ -17182,7 +17182,7 @@
         <v>326</v>
       </c>
       <c r="M131" t="n">
-        <v>1911</v>
+        <v>1933</v>
       </c>
       <c r="N131" t="inlineStr">
         <is>
@@ -17310,7 +17310,7 @@
         <v>165</v>
       </c>
       <c r="M132" t="n">
-        <v>989</v>
+        <v>1002</v>
       </c>
       <c r="N132" t="inlineStr">
         <is>
@@ -17438,7 +17438,7 @@
         <v>329</v>
       </c>
       <c r="M133" t="n">
-        <v>1899</v>
+        <v>1917</v>
       </c>
       <c r="N133" t="inlineStr">
         <is>
@@ -17566,7 +17566,7 @@
         <v>165</v>
       </c>
       <c r="M134" t="n">
-        <v>985</v>
+        <v>998</v>
       </c>
       <c r="N134" t="inlineStr">
         <is>
@@ -18718,7 +18718,7 @@
         <v>145</v>
       </c>
       <c r="M143" t="n">
-        <v>864</v>
+        <v>880</v>
       </c>
       <c r="N143" t="inlineStr">
         <is>
@@ -18846,7 +18846,7 @@
         <v>147</v>
       </c>
       <c r="M144" t="n">
-        <v>869</v>
+        <v>885</v>
       </c>
       <c r="N144" t="inlineStr">
         <is>
@@ -18974,7 +18974,7 @@
         <v>147</v>
       </c>
       <c r="M145" t="n">
-        <v>869</v>
+        <v>885</v>
       </c>
       <c r="N145" t="inlineStr">
         <is>
@@ -19102,7 +19102,7 @@
         <v>145</v>
       </c>
       <c r="M146" t="n">
-        <v>865</v>
+        <v>881</v>
       </c>
       <c r="N146" t="inlineStr">
         <is>
@@ -19230,7 +19230,7 @@
         <v>144</v>
       </c>
       <c r="M147" t="n">
-        <v>859</v>
+        <v>875</v>
       </c>
       <c r="N147" t="inlineStr">
         <is>
@@ -19358,7 +19358,7 @@
         <v>147</v>
       </c>
       <c r="M148" t="n">
-        <v>869</v>
+        <v>885</v>
       </c>
       <c r="N148" t="inlineStr">
         <is>
@@ -19486,7 +19486,7 @@
         <v>144</v>
       </c>
       <c r="M149" t="n">
-        <v>861</v>
+        <v>877</v>
       </c>
       <c r="N149" t="inlineStr">
         <is>
@@ -19614,7 +19614,7 @@
         <v>145</v>
       </c>
       <c r="M150" t="n">
-        <v>865</v>
+        <v>881</v>
       </c>
       <c r="N150" t="inlineStr">
         <is>
@@ -19742,7 +19742,7 @@
         <v>145</v>
       </c>
       <c r="M151" t="n">
-        <v>866</v>
+        <v>882</v>
       </c>
       <c r="N151" t="inlineStr">
         <is>
@@ -19870,7 +19870,7 @@
         <v>145</v>
       </c>
       <c r="M152" t="n">
-        <v>864</v>
+        <v>880</v>
       </c>
       <c r="N152" t="inlineStr">
         <is>
@@ -19998,7 +19998,7 @@
         <v>145</v>
       </c>
       <c r="M153" t="n">
-        <v>866</v>
+        <v>882</v>
       </c>
       <c r="N153" t="inlineStr">
         <is>
@@ -20126,7 +20126,7 @@
         <v>147</v>
       </c>
       <c r="M154" t="n">
-        <v>870</v>
+        <v>886</v>
       </c>
       <c r="N154" t="inlineStr">
         <is>
@@ -20254,7 +20254,7 @@
         <v>147</v>
       </c>
       <c r="M155" t="n">
-        <v>873</v>
+        <v>889</v>
       </c>
       <c r="N155" t="inlineStr">
         <is>
@@ -20382,7 +20382,7 @@
         <v>147</v>
       </c>
       <c r="M156" t="n">
-        <v>869</v>
+        <v>885</v>
       </c>
       <c r="N156" t="inlineStr">
         <is>
@@ -20510,7 +20510,7 @@
         <v>147</v>
       </c>
       <c r="M157" t="n">
-        <v>869</v>
+        <v>885</v>
       </c>
       <c r="N157" t="inlineStr">
         <is>
@@ -20638,7 +20638,7 @@
         <v>147</v>
       </c>
       <c r="M158" t="n">
-        <v>869</v>
+        <v>885</v>
       </c>
       <c r="N158" t="inlineStr">
         <is>
@@ -20766,7 +20766,7 @@
         <v>128</v>
       </c>
       <c r="M159" t="n">
-        <v>765</v>
+        <v>782</v>
       </c>
       <c r="N159" t="inlineStr">
         <is>
@@ -20894,7 +20894,7 @@
         <v>131</v>
       </c>
       <c r="M160" t="n">
-        <v>803</v>
+        <v>818</v>
       </c>
       <c r="N160" t="inlineStr">
         <is>
@@ -21278,7 +21278,7 @@
         <v>131</v>
       </c>
       <c r="M163" t="n">
-        <v>803</v>
+        <v>818</v>
       </c>
       <c r="N163" t="inlineStr">
         <is>
@@ -21534,7 +21534,7 @@
         <v>131</v>
       </c>
       <c r="M165" t="n">
-        <v>803</v>
+        <v>818</v>
       </c>
       <c r="N165" t="inlineStr">
         <is>
@@ -22046,7 +22046,7 @@
         <v>131</v>
       </c>
       <c r="M169" t="n">
-        <v>804</v>
+        <v>819</v>
       </c>
       <c r="N169" t="inlineStr">
         <is>
@@ -22174,7 +22174,7 @@
         <v>131</v>
       </c>
       <c r="M170" t="n">
-        <v>803</v>
+        <v>818</v>
       </c>
       <c r="N170" t="inlineStr">
         <is>
@@ -22302,7 +22302,7 @@
         <v>131</v>
       </c>
       <c r="M171" t="n">
-        <v>803</v>
+        <v>818</v>
       </c>
       <c r="N171" t="inlineStr">
         <is>
@@ -22430,7 +22430,7 @@
         <v>131</v>
       </c>
       <c r="M172" t="n">
-        <v>803</v>
+        <v>818</v>
       </c>
       <c r="N172" t="inlineStr">
         <is>
@@ -22558,7 +22558,7 @@
         <v>131</v>
       </c>
       <c r="M173" t="n">
-        <v>804</v>
+        <v>819</v>
       </c>
       <c r="N173" t="inlineStr">
         <is>
@@ -22814,7 +22814,7 @@
         <v>125</v>
       </c>
       <c r="M175" t="n">
-        <v>751</v>
+        <v>768</v>
       </c>
       <c r="N175" t="inlineStr">
         <is>
@@ -22942,7 +22942,7 @@
         <v>131</v>
       </c>
       <c r="M176" t="n">
-        <v>803</v>
+        <v>818</v>
       </c>
       <c r="N176" t="inlineStr">
         <is>
@@ -23070,7 +23070,7 @@
         <v>125</v>
       </c>
       <c r="M177" t="n">
-        <v>750</v>
+        <v>767</v>
       </c>
       <c r="N177" t="inlineStr">
         <is>
@@ -23198,7 +23198,7 @@
         <v>125</v>
       </c>
       <c r="M178" t="n">
-        <v>750</v>
+        <v>767</v>
       </c>
       <c r="N178" t="inlineStr">
         <is>
@@ -23838,7 +23838,7 @@
         <v>131</v>
       </c>
       <c r="M183" t="n">
-        <v>803</v>
+        <v>818</v>
       </c>
       <c r="N183" t="inlineStr">
         <is>
@@ -24094,7 +24094,7 @@
         <v>128</v>
       </c>
       <c r="M185" t="n">
-        <v>765</v>
+        <v>782</v>
       </c>
       <c r="N185" t="inlineStr">
         <is>
@@ -24222,7 +24222,7 @@
         <v>131</v>
       </c>
       <c r="M186" t="n">
-        <v>807</v>
+        <v>822</v>
       </c>
       <c r="N186" t="inlineStr">
         <is>
@@ -24478,7 +24478,7 @@
         <v>131</v>
       </c>
       <c r="M188" t="n">
-        <v>804</v>
+        <v>819</v>
       </c>
       <c r="N188" t="inlineStr">
         <is>
@@ -24606,7 +24606,7 @@
         <v>125</v>
       </c>
       <c r="M189" t="n">
-        <v>751</v>
+        <v>768</v>
       </c>
       <c r="N189" t="inlineStr">
         <is>
@@ -24862,7 +24862,7 @@
         <v>131</v>
       </c>
       <c r="M191" t="n">
-        <v>803</v>
+        <v>818</v>
       </c>
       <c r="N191" t="inlineStr">
         <is>
@@ -24990,7 +24990,7 @@
         <v>131</v>
       </c>
       <c r="M192" t="n">
-        <v>803</v>
+        <v>818</v>
       </c>
       <c r="N192" t="inlineStr">
         <is>
@@ -25246,7 +25246,7 @@
         <v>131</v>
       </c>
       <c r="M194" t="n">
-        <v>803</v>
+        <v>818</v>
       </c>
       <c r="N194" t="inlineStr">
         <is>
@@ -25374,7 +25374,7 @@
         <v>131</v>
       </c>
       <c r="M195" t="n">
-        <v>804</v>
+        <v>819</v>
       </c>
       <c r="N195" t="inlineStr">
         <is>
@@ -25502,7 +25502,7 @@
         <v>131</v>
       </c>
       <c r="M196" t="n">
-        <v>803</v>
+        <v>818</v>
       </c>
       <c r="N196" t="inlineStr">
         <is>
@@ -25630,7 +25630,7 @@
         <v>128</v>
       </c>
       <c r="M197" t="n">
-        <v>765</v>
+        <v>782</v>
       </c>
       <c r="N197" t="inlineStr">
         <is>
@@ -25758,7 +25758,7 @@
         <v>131</v>
       </c>
       <c r="M198" t="n">
-        <v>803</v>
+        <v>818</v>
       </c>
       <c r="N198" t="inlineStr">
         <is>
@@ -25886,7 +25886,7 @@
         <v>128</v>
       </c>
       <c r="M199" t="n">
-        <v>765</v>
+        <v>782</v>
       </c>
       <c r="N199" t="inlineStr">
         <is>
@@ -26142,7 +26142,7 @@
         <v>131</v>
       </c>
       <c r="M201" t="n">
-        <v>804</v>
+        <v>819</v>
       </c>
       <c r="N201" t="inlineStr">
         <is>
@@ -26270,7 +26270,7 @@
         <v>125</v>
       </c>
       <c r="M202" t="n">
-        <v>753</v>
+        <v>770</v>
       </c>
       <c r="N202" t="inlineStr">
         <is>
@@ -26398,7 +26398,7 @@
         <v>131</v>
       </c>
       <c r="M203" t="n">
-        <v>802</v>
+        <v>817</v>
       </c>
       <c r="N203" t="inlineStr">
         <is>
@@ -26654,7 +26654,7 @@
         <v>128</v>
       </c>
       <c r="M205" t="n">
-        <v>770</v>
+        <v>787</v>
       </c>
       <c r="N205" t="inlineStr">
         <is>
@@ -26910,7 +26910,7 @@
         <v>131</v>
       </c>
       <c r="M207" t="n">
-        <v>803</v>
+        <v>818</v>
       </c>
       <c r="N207" t="inlineStr">
         <is>
@@ -27166,7 +27166,7 @@
         <v>128</v>
       </c>
       <c r="M209" t="n">
-        <v>765</v>
+        <v>782</v>
       </c>
       <c r="N209" t="inlineStr">
         <is>
@@ -27294,7 +27294,7 @@
         <v>131</v>
       </c>
       <c r="M210" t="n">
-        <v>802</v>
+        <v>817</v>
       </c>
       <c r="N210" t="inlineStr">
         <is>
@@ -27678,7 +27678,7 @@
         <v>132</v>
       </c>
       <c r="M213" t="n">
-        <v>782</v>
+        <v>795</v>
       </c>
       <c r="N213" t="inlineStr">
         <is>
@@ -27806,7 +27806,7 @@
         <v>132</v>
       </c>
       <c r="M214" t="n">
-        <v>781</v>
+        <v>794</v>
       </c>
       <c r="N214" t="inlineStr">
         <is>
@@ -27934,7 +27934,7 @@
         <v>132</v>
       </c>
       <c r="M215" t="n">
-        <v>781</v>
+        <v>794</v>
       </c>
       <c r="N215" t="inlineStr">
         <is>
@@ -28062,7 +28062,7 @@
         <v>129</v>
       </c>
       <c r="M216" t="n">
-        <v>766</v>
+        <v>779</v>
       </c>
       <c r="N216" t="inlineStr">
         <is>
@@ -28190,7 +28190,7 @@
         <v>129</v>
       </c>
       <c r="M217" t="n">
-        <v>768</v>
+        <v>781</v>
       </c>
       <c r="N217" t="inlineStr">
         <is>
@@ -28318,7 +28318,7 @@
         <v>129</v>
       </c>
       <c r="M218" t="n">
-        <v>765</v>
+        <v>778</v>
       </c>
       <c r="N218" t="inlineStr">
         <is>
@@ -28446,7 +28446,7 @@
         <v>132</v>
       </c>
       <c r="M219" t="n">
-        <v>782</v>
+        <v>795</v>
       </c>
       <c r="N219" t="inlineStr">
         <is>
@@ -28574,7 +28574,7 @@
         <v>129</v>
       </c>
       <c r="M220" t="n">
-        <v>766</v>
+        <v>779</v>
       </c>
       <c r="N220" t="inlineStr">
         <is>
@@ -28702,7 +28702,7 @@
         <v>132</v>
       </c>
       <c r="M221" t="n">
-        <v>781</v>
+        <v>794</v>
       </c>
       <c r="N221" t="inlineStr">
         <is>
@@ -28830,7 +28830,7 @@
         <v>129</v>
       </c>
       <c r="M222" t="n">
-        <v>766</v>
+        <v>779</v>
       </c>
       <c r="N222" t="inlineStr">
         <is>
@@ -28958,7 +28958,7 @@
         <v>132</v>
       </c>
       <c r="M223" t="n">
-        <v>781</v>
+        <v>794</v>
       </c>
       <c r="N223" t="inlineStr">
         <is>
@@ -29086,7 +29086,7 @@
         <v>132</v>
       </c>
       <c r="M224" t="n">
-        <v>781</v>
+        <v>794</v>
       </c>
       <c r="N224" t="inlineStr">
         <is>
@@ -29214,7 +29214,7 @@
         <v>129</v>
       </c>
       <c r="M225" t="n">
-        <v>768</v>
+        <v>781</v>
       </c>
       <c r="N225" t="inlineStr">
         <is>
@@ -29342,7 +29342,7 @@
         <v>132</v>
       </c>
       <c r="M226" t="n">
-        <v>781</v>
+        <v>794</v>
       </c>
       <c r="N226" t="inlineStr">
         <is>
@@ -29470,7 +29470,7 @@
         <v>129</v>
       </c>
       <c r="M227" t="n">
-        <v>765</v>
+        <v>778</v>
       </c>
       <c r="N227" t="inlineStr">
         <is>
@@ -29598,7 +29598,7 @@
         <v>132</v>
       </c>
       <c r="M228" t="n">
-        <v>781</v>
+        <v>794</v>
       </c>
       <c r="N228" t="inlineStr">
         <is>
@@ -29726,7 +29726,7 @@
         <v>132</v>
       </c>
       <c r="M229" t="n">
-        <v>782</v>
+        <v>795</v>
       </c>
       <c r="N229" t="inlineStr">
         <is>
@@ -29854,7 +29854,7 @@
         <v>132</v>
       </c>
       <c r="M230" t="n">
-        <v>782</v>
+        <v>795</v>
       </c>
       <c r="N230" t="inlineStr">
         <is>
@@ -29982,7 +29982,7 @@
         <v>129</v>
       </c>
       <c r="M231" t="n">
-        <v>766</v>
+        <v>779</v>
       </c>
       <c r="N231" t="inlineStr">
         <is>
@@ -30110,7 +30110,7 @@
         <v>132</v>
       </c>
       <c r="M232" t="n">
-        <v>781</v>
+        <v>794</v>
       </c>
       <c r="N232" t="inlineStr">
         <is>
@@ -30238,7 +30238,7 @@
         <v>129</v>
       </c>
       <c r="M233" t="n">
-        <v>766</v>
+        <v>779</v>
       </c>
       <c r="N233" t="inlineStr">
         <is>
@@ -30366,7 +30366,7 @@
         <v>144</v>
       </c>
       <c r="M234" t="n">
-        <v>847</v>
+        <v>861</v>
       </c>
       <c r="N234" t="inlineStr">
         <is>
@@ -30494,7 +30494,7 @@
         <v>130</v>
       </c>
       <c r="M235" t="n">
-        <v>775</v>
+        <v>789</v>
       </c>
       <c r="N235" t="inlineStr">
         <is>
@@ -30622,7 +30622,7 @@
         <v>144</v>
       </c>
       <c r="M236" t="n">
-        <v>851</v>
+        <v>865</v>
       </c>
       <c r="N236" t="inlineStr">
         <is>
@@ -30750,7 +30750,7 @@
         <v>143</v>
       </c>
       <c r="M237" t="n">
-        <v>845</v>
+        <v>859</v>
       </c>
       <c r="N237" t="inlineStr">
         <is>
@@ -30878,7 +30878,7 @@
         <v>146</v>
       </c>
       <c r="M238" t="n">
-        <v>854</v>
+        <v>868</v>
       </c>
       <c r="N238" t="inlineStr">
         <is>
@@ -31006,7 +31006,7 @@
         <v>144</v>
       </c>
       <c r="M239" t="n">
-        <v>849</v>
+        <v>863</v>
       </c>
       <c r="N239" t="inlineStr">
         <is>
@@ -31134,7 +31134,7 @@
         <v>144</v>
       </c>
       <c r="M240" t="n">
-        <v>851</v>
+        <v>865</v>
       </c>
       <c r="N240" t="inlineStr">
         <is>
@@ -31262,7 +31262,7 @@
         <v>144</v>
       </c>
       <c r="M241" t="n">
-        <v>849</v>
+        <v>863</v>
       </c>
       <c r="N241" t="inlineStr">
         <is>
@@ -31390,7 +31390,7 @@
         <v>130</v>
       </c>
       <c r="M242" t="n">
-        <v>775</v>
+        <v>789</v>
       </c>
       <c r="N242" t="inlineStr">
         <is>
@@ -31518,7 +31518,7 @@
         <v>146</v>
       </c>
       <c r="M243" t="n">
-        <v>854</v>
+        <v>868</v>
       </c>
       <c r="N243" t="inlineStr">
         <is>
@@ -31646,7 +31646,7 @@
         <v>146</v>
       </c>
       <c r="M244" t="n">
-        <v>853</v>
+        <v>867</v>
       </c>
       <c r="N244" t="inlineStr">
         <is>
@@ -31774,7 +31774,7 @@
         <v>124</v>
       </c>
       <c r="M245" t="n">
-        <v>745</v>
+        <v>759</v>
       </c>
       <c r="N245" t="inlineStr">
         <is>
@@ -31902,7 +31902,7 @@
         <v>144</v>
       </c>
       <c r="M246" t="n">
-        <v>847</v>
+        <v>861</v>
       </c>
       <c r="N246" t="inlineStr">
         <is>
@@ -32030,7 +32030,7 @@
         <v>146</v>
       </c>
       <c r="M247" t="n">
-        <v>854</v>
+        <v>868</v>
       </c>
       <c r="N247" t="inlineStr">
         <is>
@@ -32158,7 +32158,7 @@
         <v>110</v>
       </c>
       <c r="M248" t="n">
-        <v>680</v>
+        <v>693</v>
       </c>
       <c r="N248" t="inlineStr">
         <is>
@@ -32286,7 +32286,7 @@
         <v>146</v>
       </c>
       <c r="M249" t="n">
-        <v>854</v>
+        <v>868</v>
       </c>
       <c r="N249" t="inlineStr">
         <is>
@@ -32414,7 +32414,7 @@
         <v>144</v>
       </c>
       <c r="M250" t="n">
-        <v>851</v>
+        <v>865</v>
       </c>
       <c r="N250" t="inlineStr">
         <is>
@@ -32542,7 +32542,7 @@
         <v>146</v>
       </c>
       <c r="M251" t="n">
-        <v>854</v>
+        <v>868</v>
       </c>
       <c r="N251" t="inlineStr">
         <is>
@@ -32670,7 +32670,7 @@
         <v>129</v>
       </c>
       <c r="M252" t="n">
-        <v>774</v>
+        <v>787</v>
       </c>
       <c r="N252" t="inlineStr">
         <is>
@@ -32798,7 +32798,7 @@
         <v>129</v>
       </c>
       <c r="M253" t="n">
-        <v>773</v>
+        <v>786</v>
       </c>
       <c r="N253" t="inlineStr">
         <is>
@@ -32926,7 +32926,7 @@
         <v>129</v>
       </c>
       <c r="M254" t="n">
-        <v>775</v>
+        <v>788</v>
       </c>
       <c r="N254" t="inlineStr">
         <is>
@@ -33054,7 +33054,7 @@
         <v>129</v>
       </c>
       <c r="M255" t="n">
-        <v>776</v>
+        <v>789</v>
       </c>
       <c r="N255" t="inlineStr">
         <is>
@@ -33310,7 +33310,7 @@
         <v>132</v>
       </c>
       <c r="M257" t="n">
-        <v>793</v>
+        <v>806</v>
       </c>
       <c r="N257" t="inlineStr">
         <is>
@@ -33438,7 +33438,7 @@
         <v>110</v>
       </c>
       <c r="M258" t="n">
-        <v>684</v>
+        <v>697</v>
       </c>
       <c r="N258" t="inlineStr">
         <is>
@@ -33566,7 +33566,7 @@
         <v>132</v>
       </c>
       <c r="M259" t="n">
-        <v>792</v>
+        <v>805</v>
       </c>
       <c r="N259" t="inlineStr">
         <is>
@@ -33694,7 +33694,7 @@
         <v>129</v>
       </c>
       <c r="M260" t="n">
-        <v>774</v>
+        <v>787</v>
       </c>
       <c r="N260" t="inlineStr">
         <is>
@@ -33822,7 +33822,7 @@
         <v>132</v>
       </c>
       <c r="M261" t="n">
-        <v>790</v>
+        <v>803</v>
       </c>
       <c r="N261" t="inlineStr">
         <is>
@@ -33950,7 +33950,7 @@
         <v>132</v>
       </c>
       <c r="M262" t="n">
-        <v>792</v>
+        <v>805</v>
       </c>
       <c r="N262" t="inlineStr">
         <is>
@@ -34078,7 +34078,7 @@
         <v>132</v>
       </c>
       <c r="M263" t="n">
-        <v>793</v>
+        <v>806</v>
       </c>
       <c r="N263" t="inlineStr">
         <is>
@@ -34206,7 +34206,7 @@
         <v>129</v>
       </c>
       <c r="M264" t="n">
-        <v>776</v>
+        <v>789</v>
       </c>
       <c r="N264" t="inlineStr">
         <is>
@@ -34334,7 +34334,7 @@
         <v>132</v>
       </c>
       <c r="M265" t="n">
-        <v>792</v>
+        <v>805</v>
       </c>
       <c r="N265" t="inlineStr">
         <is>
@@ -34462,7 +34462,7 @@
         <v>129</v>
       </c>
       <c r="M266" t="n">
-        <v>774</v>
+        <v>787</v>
       </c>
       <c r="N266" t="inlineStr">
         <is>
@@ -34590,7 +34590,7 @@
         <v>132</v>
       </c>
       <c r="M267" t="n">
-        <v>793</v>
+        <v>806</v>
       </c>
       <c r="N267" t="inlineStr">
         <is>
@@ -34718,7 +34718,7 @@
         <v>129</v>
       </c>
       <c r="M268" t="n">
-        <v>776</v>
+        <v>789</v>
       </c>
       <c r="N268" t="inlineStr">
         <is>
@@ -34974,7 +34974,7 @@
         <v>129</v>
       </c>
       <c r="M270" t="n">
-        <v>776</v>
+        <v>789</v>
       </c>
       <c r="N270" t="inlineStr">
         <is>
@@ -35102,7 +35102,7 @@
         <v>129</v>
       </c>
       <c r="M271" t="n">
-        <v>773</v>
+        <v>786</v>
       </c>
       <c r="N271" t="inlineStr">
         <is>
@@ -35230,7 +35230,7 @@
         <v>129</v>
       </c>
       <c r="M272" t="n">
-        <v>776</v>
+        <v>789</v>
       </c>
       <c r="N272" t="inlineStr">
         <is>

</xml_diff>